<commit_message>
modifiche di ottimizzazione codice
</commit_message>
<xml_diff>
--- a/RISULTATI AUTOSAM/autoSamKlnmJ.xlsx
+++ b/RISULTATI AUTOSAM/autoSamKlnmJ.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28827"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\OneDrive - Politecnico di Milano\Documenti\POLIMI\Tesi\distillation\RISULTATI AUTOSAM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A25DB167-3018-4500-B48E-C328132456E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BD06172-E2FA-4A2D-942D-9AB72DF827BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1404" yWindow="1104" windowWidth="21600" windowHeight="11232" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Worksheet" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -74,7 +75,7 @@
     <t>Iou</t>
   </si>
   <si>
-    <t>MASCHERE CON REFINING</t>
+    <t xml:space="preserve">MASCHERE CON REFINING  che non viene considerto nel conteggio del tempo </t>
   </si>
 </sst>
 </file>
@@ -166,7 +167,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -178,8 +179,7 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -791,13 +791,13 @@
       <c r="D7" t="s">
         <v>12</v>
       </c>
-      <c r="G7" s="9" t="s">
+      <c r="G7" t="s">
         <v>0</v>
       </c>
-      <c r="H7" s="9" t="s">
+      <c r="H7" t="s">
         <v>1</v>
       </c>
-      <c r="I7" s="9" t="s">
+      <c r="I7" t="s">
         <v>2</v>
       </c>
       <c r="S7" s="2" t="s">
@@ -814,13 +814,13 @@
       <c r="D8">
         <v>0.80501519509857</v>
       </c>
-      <c r="G8" s="9">
+      <c r="G8">
         <v>528.47409248352005</v>
       </c>
-      <c r="H8" s="9">
+      <c r="H8">
         <v>0</v>
       </c>
-      <c r="I8" s="9">
+      <c r="I8">
         <v>0.80508674277821002</v>
       </c>
       <c r="P8" s="3" t="s">
@@ -840,13 +840,13 @@
       <c r="D9">
         <v>0.83156960747603004</v>
       </c>
-      <c r="G9" s="9">
+      <c r="G9">
         <v>41.107177734375</v>
       </c>
-      <c r="H9" s="9">
+      <c r="H9">
         <v>1</v>
       </c>
-      <c r="I9" s="9">
+      <c r="I9">
         <v>0.84273808583795995</v>
       </c>
       <c r="O9" t="s">
@@ -878,13 +878,13 @@
       <c r="D10">
         <v>0.83700486448922995</v>
       </c>
-      <c r="G10" s="9">
+      <c r="G10">
         <v>26.023149490356001</v>
       </c>
-      <c r="H10" s="9">
+      <c r="H10">
         <v>2</v>
       </c>
-      <c r="I10" s="9">
+      <c r="I10">
         <v>0.79840175431664995</v>
       </c>
       <c r="O10">
@@ -916,13 +916,13 @@
       <c r="D11">
         <v>0.80355264580690999</v>
       </c>
-      <c r="G11" s="9">
+      <c r="G11">
         <v>24.88899230957</v>
       </c>
-      <c r="H11" s="9">
+      <c r="H11">
         <v>3</v>
       </c>
-      <c r="I11" s="9">
+      <c r="I11">
         <v>0.80840322709482004</v>
       </c>
       <c r="O11">
@@ -954,13 +954,13 @@
       <c r="D12">
         <v>0.82161024099774005</v>
       </c>
-      <c r="G12" s="9">
+      <c r="G12">
         <v>25.722503662108998</v>
       </c>
-      <c r="H12" s="9">
+      <c r="H12">
         <v>4</v>
       </c>
-      <c r="I12" s="9">
+      <c r="I12">
         <v>0.82876194508286005</v>
       </c>
       <c r="O12">
@@ -992,13 +992,13 @@
       <c r="D13">
         <v>0.83015130244891999</v>
       </c>
-      <c r="G13" s="9">
+      <c r="G13">
         <v>25.054693222046001</v>
       </c>
-      <c r="H13" s="9">
+      <c r="H13">
         <v>5</v>
       </c>
-      <c r="I13" s="9">
+      <c r="I13">
         <v>0.83003563320353002</v>
       </c>
       <c r="O13">
@@ -1030,13 +1030,13 @@
       <c r="D14">
         <v>0.84068800700125002</v>
       </c>
-      <c r="G14" s="9">
+      <c r="G14">
         <v>26.760339736938</v>
       </c>
-      <c r="H14" s="9">
+      <c r="H14">
         <v>6</v>
       </c>
-      <c r="I14" s="9">
+      <c r="I14">
         <v>0.83660704799008001</v>
       </c>
       <c r="O14">
@@ -1068,13 +1068,13 @@
       <c r="D15">
         <v>0.79002643829173003</v>
       </c>
-      <c r="G15" s="9">
+      <c r="G15">
         <v>26.602268218993999</v>
       </c>
-      <c r="H15" s="9">
+      <c r="H15">
         <v>7</v>
       </c>
-      <c r="I15" s="9">
+      <c r="I15">
         <v>0.83560081239741002</v>
       </c>
       <c r="O15">
@@ -1106,13 +1106,13 @@
       <c r="D16">
         <v>0.85129722642172001</v>
       </c>
-      <c r="G16" s="9">
+      <c r="G16">
         <v>25.592088699341002</v>
       </c>
-      <c r="H16" s="9">
+      <c r="H16">
         <v>8</v>
       </c>
-      <c r="I16" s="9">
+      <c r="I16">
         <v>0.82139931048468995</v>
       </c>
       <c r="O16">
@@ -1144,13 +1144,13 @@
       <c r="D17">
         <v>0.85497591208393997</v>
       </c>
-      <c r="G17" s="9">
+      <c r="G17">
         <v>27.924776077271002</v>
       </c>
-      <c r="H17" s="9">
+      <c r="H17">
         <v>9</v>
       </c>
-      <c r="I17" s="9">
+      <c r="I17">
         <v>0.78561886912832002</v>
       </c>
       <c r="O17">
@@ -1182,13 +1182,13 @@
       <c r="D18">
         <v>0.82138621637541998</v>
       </c>
-      <c r="G18" s="9">
+      <c r="G18">
         <v>25.401830673218001</v>
       </c>
-      <c r="H18" s="9">
+      <c r="H18">
         <v>10</v>
       </c>
-      <c r="I18" s="9">
+      <c r="I18">
         <v>0.84537783828212998</v>
       </c>
       <c r="O18">
@@ -1220,13 +1220,13 @@
       <c r="D19">
         <v>0.84679539612058996</v>
       </c>
-      <c r="G19" s="9">
+      <c r="G19">
         <v>26.759386062621999</v>
       </c>
-      <c r="H19" s="9">
+      <c r="H19">
         <v>11</v>
       </c>
-      <c r="I19" s="9">
+      <c r="I19">
         <v>0.80488222628213002</v>
       </c>
       <c r="O19">
@@ -1258,13 +1258,13 @@
       <c r="D20">
         <v>0.83183630846531997</v>
       </c>
-      <c r="G20" s="9">
+      <c r="G20">
         <v>27.643442153931002</v>
       </c>
-      <c r="H20" s="9">
+      <c r="H20">
         <v>12</v>
       </c>
-      <c r="I20" s="9">
+      <c r="I20">
         <v>0.84037478462699999</v>
       </c>
       <c r="O20">
@@ -1296,13 +1296,13 @@
       <c r="D21">
         <v>0.83561472331191</v>
       </c>
-      <c r="G21" s="9">
+      <c r="G21">
         <v>25.014162063598999</v>
       </c>
-      <c r="H21" s="9">
+      <c r="H21">
         <v>13</v>
       </c>
-      <c r="I21" s="9">
+      <c r="I21">
         <v>0.81227416117006002</v>
       </c>
       <c r="O21">
@@ -1334,13 +1334,13 @@
       <c r="D22">
         <v>0.82940149451777001</v>
       </c>
-      <c r="G22" s="9">
+      <c r="G22">
         <v>28.335809707641999</v>
       </c>
-      <c r="H22" s="9">
+      <c r="H22">
         <v>14</v>
       </c>
-      <c r="I22" s="9">
+      <c r="I22">
         <v>0.82108194981899996</v>
       </c>
       <c r="O22">
@@ -1372,13 +1372,13 @@
       <c r="D23">
         <v>0.83377762294958002</v>
       </c>
-      <c r="G23" s="9">
+      <c r="G23">
         <v>25.141954421996999</v>
       </c>
-      <c r="H23" s="9">
+      <c r="H23">
         <v>15</v>
       </c>
-      <c r="I23" s="9">
+      <c r="I23">
         <v>0.81903634312775997</v>
       </c>
       <c r="O23">
@@ -1410,13 +1410,13 @@
       <c r="D24">
         <v>0.86239385231345</v>
       </c>
-      <c r="G24" s="9">
+      <c r="G24">
         <v>25.549650192261002</v>
       </c>
-      <c r="H24" s="9">
+      <c r="H24">
         <v>16</v>
       </c>
-      <c r="I24" s="9">
+      <c r="I24">
         <v>0.82944220575603</v>
       </c>
       <c r="O24">
@@ -1448,13 +1448,13 @@
       <c r="D25">
         <v>0.81428391242089004</v>
       </c>
-      <c r="G25" s="9">
+      <c r="G25">
         <v>26.713132858276001</v>
       </c>
-      <c r="H25" s="9">
+      <c r="H25">
         <v>17</v>
       </c>
-      <c r="I25" s="9">
+      <c r="I25">
         <v>0.82161971038716997</v>
       </c>
       <c r="O25">
@@ -1486,13 +1486,13 @@
       <c r="D26">
         <v>0.82871549853715998</v>
       </c>
-      <c r="G26" s="9">
+      <c r="G26">
         <v>26.226758956908998</v>
       </c>
-      <c r="H26" s="9">
+      <c r="H26">
         <v>18</v>
       </c>
-      <c r="I26" s="9">
+      <c r="I26">
         <v>0.81860796579301998</v>
       </c>
       <c r="O26">
@@ -1524,13 +1524,13 @@
       <c r="D27">
         <v>0.83195290265899002</v>
       </c>
-      <c r="G27" s="9">
+      <c r="G27">
         <v>26.793003082275</v>
       </c>
-      <c r="H27" s="9">
+      <c r="H27">
         <v>19</v>
       </c>
-      <c r="I27" s="9">
+      <c r="I27">
         <v>0.83181360716149999</v>
       </c>
       <c r="O27">
@@ -1562,13 +1562,13 @@
       <c r="D28">
         <v>0.83431069806111002</v>
       </c>
-      <c r="G28" s="9">
+      <c r="G28">
         <v>25.728464126586999</v>
       </c>
-      <c r="H28" s="9">
+      <c r="H28">
         <v>20</v>
       </c>
-      <c r="I28" s="9">
+      <c r="I28">
         <v>0.81426137428973999</v>
       </c>
       <c r="O28">
@@ -1600,13 +1600,13 @@
       <c r="D29">
         <v>0.81423843219095005</v>
       </c>
-      <c r="G29" s="9">
+      <c r="G29">
         <v>25.140285491943001</v>
       </c>
-      <c r="H29" s="9">
+      <c r="H29">
         <v>21</v>
       </c>
-      <c r="I29" s="9">
+      <c r="I29">
         <v>0.86238425477509995</v>
       </c>
       <c r="O29">
@@ -1638,13 +1638,13 @@
       <c r="D30">
         <v>0.85345374961160003</v>
       </c>
-      <c r="G30" s="9">
+      <c r="G30">
         <v>30.47251701355</v>
       </c>
-      <c r="H30" s="9">
+      <c r="H30">
         <v>22</v>
       </c>
-      <c r="I30" s="9">
+      <c r="I30">
         <v>0.83388109819130996</v>
       </c>
       <c r="O30">
@@ -1676,13 +1676,13 @@
       <c r="D31">
         <v>0.81695087342604</v>
       </c>
-      <c r="G31" s="9">
+      <c r="G31">
         <v>26.216745376586999</v>
       </c>
-      <c r="H31" s="9">
+      <c r="H31">
         <v>23</v>
       </c>
-      <c r="I31" s="9">
+      <c r="I31">
         <v>0.83998554449083995</v>
       </c>
       <c r="O31">
@@ -1714,13 +1714,13 @@
       <c r="D32">
         <v>0.85760498332431001</v>
       </c>
-      <c r="G32" s="9">
+      <c r="G32">
         <v>25.721788406371999</v>
       </c>
-      <c r="H32" s="9">
+      <c r="H32">
         <v>24</v>
       </c>
-      <c r="I32" s="9">
+      <c r="I32">
         <v>0.80355457691097998</v>
       </c>
       <c r="O32">
@@ -1752,13 +1752,13 @@
       <c r="D33">
         <v>0.79844111196727996</v>
       </c>
-      <c r="G33" s="9">
+      <c r="G33">
         <v>25.134086608886999</v>
       </c>
-      <c r="H33" s="9">
+      <c r="H33">
         <v>25</v>
       </c>
-      <c r="I33" s="9">
+      <c r="I33">
         <v>0.85496394897393002</v>
       </c>
       <c r="O33">
@@ -1790,13 +1790,13 @@
       <c r="D34">
         <v>0.82350776206635001</v>
       </c>
-      <c r="G34" s="9">
+      <c r="G34">
         <v>25.261402130126999</v>
       </c>
-      <c r="H34" s="9">
+      <c r="H34">
         <v>26</v>
       </c>
-      <c r="I34" s="9">
+      <c r="I34">
         <v>0.77217953346054002</v>
       </c>
       <c r="O34">
@@ -1828,13 +1828,13 @@
       <c r="D35">
         <v>0.83385021209853005</v>
       </c>
-      <c r="G35" s="9">
+      <c r="G35">
         <v>28.221130371093999</v>
       </c>
-      <c r="H35" s="9">
+      <c r="H35">
         <v>27</v>
       </c>
-      <c r="I35" s="9">
+      <c r="I35">
         <v>0.79001832838629005</v>
       </c>
       <c r="O35">
@@ -1866,13 +1866,13 @@
       <c r="D36">
         <v>0.80492300665535998</v>
       </c>
-      <c r="G36" s="9">
+      <c r="G36">
         <v>25.766611099243001</v>
       </c>
-      <c r="H36" s="9">
+      <c r="H36">
         <v>28</v>
       </c>
-      <c r="I36" s="9">
+      <c r="I36">
         <v>0.79927674700527995</v>
       </c>
       <c r="O36">
@@ -1904,13 +1904,13 @@
       <c r="D37">
         <v>0.82106133657881997</v>
       </c>
-      <c r="G37" s="9">
+      <c r="G37">
         <v>25.092840194701999</v>
       </c>
-      <c r="H37" s="9">
+      <c r="H37">
         <v>29</v>
       </c>
-      <c r="I37" s="9">
+      <c r="I37">
         <v>0.83702526147538003</v>
       </c>
       <c r="O37">
@@ -1942,13 +1942,13 @@
       <c r="D38">
         <v>0.80388964962511</v>
       </c>
-      <c r="G38" s="9">
+      <c r="G38">
         <v>25.310277938843001</v>
       </c>
-      <c r="H38" s="9">
+      <c r="H38">
         <v>30</v>
       </c>
-      <c r="I38" s="9">
+      <c r="I38">
         <v>0.85098334259135999</v>
       </c>
       <c r="O38">
@@ -1980,13 +1980,13 @@
       <c r="D39">
         <v>0.81850359096991998</v>
       </c>
-      <c r="G39" s="9">
+      <c r="G39">
         <v>25.156736373901001</v>
       </c>
-      <c r="H39" s="9">
+      <c r="H39">
         <v>31</v>
       </c>
-      <c r="I39" s="9">
+      <c r="I39">
         <v>0.82136265462399005</v>
       </c>
       <c r="O39">
@@ -2018,13 +2018,13 @@
       <c r="D40">
         <v>0.82936838305176996</v>
       </c>
-      <c r="G40" s="9">
+      <c r="G40">
         <v>26.094436645508001</v>
       </c>
-      <c r="H40" s="9">
+      <c r="H40">
         <v>32</v>
       </c>
-      <c r="I40" s="9">
+      <c r="I40">
         <v>0.79751915034020004</v>
       </c>
       <c r="O40">
@@ -2056,13 +2056,13 @@
       <c r="D41">
         <v>0.84725495908259996</v>
       </c>
-      <c r="G41" s="9">
+      <c r="G41">
         <v>27.351856231688998</v>
       </c>
-      <c r="H41" s="9">
+      <c r="H41">
         <v>33</v>
       </c>
-      <c r="I41" s="9">
+      <c r="I41">
         <v>0.86610031559515999</v>
       </c>
       <c r="O41">
@@ -2094,13 +2094,13 @@
       <c r="D42">
         <v>0.78727292368074997</v>
       </c>
-      <c r="G42" s="9">
+      <c r="G42">
         <v>25.675058364868001</v>
       </c>
-      <c r="H42" s="9">
+      <c r="H42">
         <v>34</v>
       </c>
-      <c r="I42" s="9">
+      <c r="I42">
         <v>0.85762122781807004</v>
       </c>
       <c r="O42">
@@ -2132,13 +2132,13 @@
       <c r="D43">
         <v>0.81906255250042004</v>
       </c>
-      <c r="G43" s="9">
+      <c r="G43">
         <v>25.218963623046999</v>
       </c>
-      <c r="H43" s="9">
+      <c r="H43">
         <v>35</v>
       </c>
-      <c r="I43" s="9">
+      <c r="I43">
         <v>0.80393565067508999</v>
       </c>
       <c r="O43">
@@ -2170,13 +2170,13 @@
       <c r="D44">
         <v>0.77214830858086003</v>
       </c>
-      <c r="G44" s="9">
+      <c r="G44">
         <v>25.39324760437</v>
       </c>
-      <c r="H44" s="9">
+      <c r="H44">
         <v>36</v>
       </c>
-      <c r="I44" s="9">
+      <c r="I44">
         <v>0.85131659083581002</v>
       </c>
       <c r="O44">
@@ -2208,13 +2208,13 @@
       <c r="D45">
         <v>0.85009629443553003</v>
       </c>
-      <c r="G45" s="9">
+      <c r="G45">
         <v>26.743173599243001</v>
       </c>
-      <c r="H45" s="9">
+      <c r="H45">
         <v>37</v>
       </c>
-      <c r="I45" s="9">
+      <c r="I45">
         <v>0.85349229937854998</v>
       </c>
       <c r="O45">
@@ -2246,13 +2246,13 @@
       <c r="D46">
         <v>0.84273542311199001</v>
       </c>
-      <c r="G46" s="9">
+      <c r="G46">
         <v>26.322364807128999</v>
       </c>
-      <c r="H46" s="9">
+      <c r="H46">
         <v>38</v>
       </c>
-      <c r="I46" s="9">
+      <c r="I46">
         <v>0.84925958451940997</v>
       </c>
       <c r="O46">
@@ -2284,13 +2284,13 @@
       <c r="D47">
         <v>0.83657755677390999</v>
       </c>
-      <c r="G47" s="9">
+      <c r="G47">
         <v>25.263071060181002</v>
       </c>
-      <c r="H47" s="9">
+      <c r="H47">
         <v>39</v>
       </c>
-      <c r="I47" s="9">
+      <c r="I47">
         <v>0.83855155190867003</v>
       </c>
       <c r="O47">
@@ -2322,13 +2322,13 @@
       <c r="D48">
         <v>0.80120089705563002</v>
       </c>
-      <c r="G48" s="9">
+      <c r="G48">
         <v>25.878190994263001</v>
       </c>
-      <c r="H48" s="9">
+      <c r="H48">
         <v>40</v>
       </c>
-      <c r="I48" s="9">
+      <c r="I48">
         <v>0.78727100868704003</v>
       </c>
       <c r="O48">
@@ -2360,13 +2360,13 @@
       <c r="D49">
         <v>0.80837433701834005</v>
       </c>
-      <c r="G49" s="9">
+      <c r="G49">
         <v>26.958227157593001</v>
       </c>
-      <c r="H49" s="9">
+      <c r="H49">
         <v>41</v>
       </c>
-      <c r="I49" s="9">
+      <c r="I49">
         <v>0.82357703829648998</v>
       </c>
       <c r="O49">
@@ -2398,13 +2398,13 @@
       <c r="D50">
         <v>0.84840711764411003</v>
       </c>
-      <c r="G50" s="9">
+      <c r="G50">
         <v>27.319192886353001</v>
       </c>
-      <c r="H50" s="9">
+      <c r="H50">
         <v>42</v>
       </c>
-      <c r="I50" s="9">
+      <c r="I50">
         <v>0.85017648271241997</v>
       </c>
       <c r="O50">
@@ -2436,13 +2436,13 @@
       <c r="D51">
         <v>0.80235392776348002</v>
       </c>
-      <c r="G51" s="9">
+      <c r="G51">
         <v>26.452541351318001</v>
       </c>
-      <c r="H51" s="9">
+      <c r="H51">
         <v>43</v>
       </c>
-      <c r="I51" s="9">
+      <c r="I51">
         <v>0.83208686249774999</v>
       </c>
       <c r="O51">
@@ -2474,13 +2474,13 @@
       <c r="D52">
         <v>0.81224804168987996</v>
       </c>
-      <c r="G52" s="9">
+      <c r="G52">
         <v>25.809764862061002</v>
       </c>
-      <c r="H52" s="9">
+      <c r="H52">
         <v>44</v>
       </c>
-      <c r="I52" s="9">
+      <c r="I52">
         <v>0.84061151539223</v>
       </c>
       <c r="O52">
@@ -2512,13 +2512,13 @@
       <c r="D53">
         <v>0.80114879649891002</v>
       </c>
-      <c r="G53" s="9">
+      <c r="G53">
         <v>27.360200881958001</v>
       </c>
-      <c r="H53" s="9">
+      <c r="H53">
         <v>45</v>
       </c>
-      <c r="I53" s="9">
+      <c r="I53">
         <v>0.81698497898722999</v>
       </c>
       <c r="O53">
@@ -2550,13 +2550,13 @@
       <c r="D54">
         <v>0.83815839384415003</v>
       </c>
-      <c r="G54" s="9">
+      <c r="G54">
         <v>25.617599487305</v>
       </c>
-      <c r="H54" s="9">
+      <c r="H54">
         <v>46</v>
       </c>
-      <c r="I54" s="9">
+      <c r="I54">
         <v>0.77950528762138005</v>
       </c>
       <c r="O54">
@@ -2588,13 +2588,13 @@
       <c r="D55">
         <v>0.78563666995643999</v>
       </c>
-      <c r="G55" s="9">
+      <c r="G55">
         <v>26.685476303101002</v>
       </c>
-      <c r="H55" s="9">
+      <c r="H55">
         <v>47</v>
       </c>
-      <c r="I55" s="9">
+      <c r="I55">
         <v>0.83016557608467001</v>
       </c>
       <c r="O55">
@@ -2626,13 +2626,13 @@
       <c r="D56">
         <v>0.84477495001891001</v>
       </c>
-      <c r="G56" s="9">
+      <c r="G56">
         <v>28.676509857178001</v>
       </c>
-      <c r="H56" s="9">
+      <c r="H56">
         <v>48</v>
       </c>
-      <c r="I56" s="9">
+      <c r="I56">
         <v>0.82935022837778005</v>
       </c>
       <c r="O56">
@@ -2664,13 +2664,13 @@
       <c r="D57">
         <v>0.86608796908908003</v>
       </c>
-      <c r="G57" s="9">
+      <c r="G57">
         <v>25.192975997925</v>
       </c>
-      <c r="H57" s="9">
+      <c r="H57">
         <v>49</v>
       </c>
-      <c r="I57" s="9">
+      <c r="I57">
         <v>0.81680529446604999</v>
       </c>
       <c r="O57">
@@ -2702,13 +2702,13 @@
       <c r="D58">
         <v>0.80185813329357003</v>
       </c>
-      <c r="G58" s="9">
+      <c r="G58">
         <v>27.429580688476999</v>
       </c>
-      <c r="H58" s="9">
+      <c r="H58">
         <v>50</v>
       </c>
-      <c r="I58" s="9">
+      <c r="I58">
         <v>0.83156009605601</v>
       </c>
       <c r="O58">
@@ -2740,13 +2740,13 @@
       <c r="D59">
         <v>0.79930134593650004</v>
       </c>
-      <c r="G59" s="9">
+      <c r="G59">
         <v>25.159120559691999</v>
       </c>
-      <c r="H59" s="9">
+      <c r="H59">
         <v>51</v>
       </c>
-      <c r="I59" s="9">
+      <c r="I59">
         <v>0.83389627699858004</v>
       </c>
       <c r="O59">
@@ -2778,13 +2778,13 @@
       <c r="D60">
         <v>0.79742286427679998</v>
       </c>
-      <c r="G60" s="9">
+      <c r="G60">
         <v>27.221441268921001</v>
       </c>
-      <c r="H60" s="9">
+      <c r="H60">
         <v>52</v>
       </c>
-      <c r="I60" s="9">
+      <c r="I60">
         <v>0.80253137402123997</v>
       </c>
       <c r="O60">
@@ -2816,13 +2816,13 @@
       <c r="D61">
         <v>0.84512052602514998</v>
       </c>
-      <c r="G61" s="9">
+      <c r="G61">
         <v>25.235891342163001</v>
       </c>
-      <c r="H61" s="9">
+      <c r="H61">
         <v>53</v>
       </c>
-      <c r="I61" s="9">
+      <c r="I61">
         <v>0.85090146908397002</v>
       </c>
       <c r="O61">
@@ -2854,13 +2854,13 @@
       <c r="D62">
         <v>0.84817764188121003</v>
       </c>
-      <c r="G62" s="9">
+      <c r="G62">
         <v>27.469873428345</v>
       </c>
-      <c r="H62" s="9">
+      <c r="H62">
         <v>54</v>
       </c>
-      <c r="I62" s="9">
+      <c r="I62">
         <v>0.80126779158301997</v>
       </c>
       <c r="O62">
@@ -2892,13 +2892,13 @@
       <c r="D63">
         <v>0.85096045674428999</v>
       </c>
-      <c r="G63" s="9">
+      <c r="G63">
         <v>25.155067443848001</v>
       </c>
-      <c r="H63" s="9">
+      <c r="H63">
         <v>55</v>
       </c>
-      <c r="I63" s="9">
+      <c r="I63">
         <v>0.84720300323761999</v>
       </c>
       <c r="O63">
@@ -2930,13 +2930,13 @@
       <c r="D64">
         <v>0.82904783523876002</v>
       </c>
-      <c r="G64" s="9">
+      <c r="G64">
         <v>25.663137435913001</v>
       </c>
-      <c r="H64" s="9">
+      <c r="H64">
         <v>56</v>
       </c>
-      <c r="I64" s="9">
+      <c r="I64">
         <v>0.80387419836597995</v>
       </c>
       <c r="O64">
@@ -2968,13 +2968,13 @@
       <c r="D65">
         <v>0.83828739397936003</v>
       </c>
-      <c r="G65" s="9">
+      <c r="G65">
         <v>27.061223983765</v>
       </c>
-      <c r="H65" s="9">
+      <c r="H65">
         <v>57</v>
       </c>
-      <c r="I65" s="9">
+      <c r="I65">
         <v>0.84679651498221997</v>
       </c>
       <c r="O65">
@@ -3006,13 +3006,13 @@
       <c r="D66">
         <v>0.84036168167740999</v>
       </c>
-      <c r="G66" s="9">
+      <c r="G66">
         <v>25.658845901488998</v>
       </c>
-      <c r="H66" s="9">
+      <c r="H66">
         <v>58</v>
       </c>
-      <c r="I66" s="9">
+      <c r="I66">
         <v>0.80451867223374995</v>
       </c>
       <c r="O66">
@@ -3044,13 +3044,13 @@
       <c r="D67">
         <v>0.83854694390135998</v>
       </c>
-      <c r="G67" s="9">
+      <c r="G67">
         <v>25.208234786986999</v>
       </c>
-      <c r="H67" s="9">
+      <c r="H67">
         <v>59</v>
       </c>
-      <c r="I67" s="9">
+      <c r="I67">
         <v>0.84843584453243004</v>
       </c>
       <c r="O67">
@@ -3082,13 +3082,13 @@
       <c r="D68">
         <v>0.82851264384315004</v>
       </c>
-      <c r="G68" s="9">
+      <c r="G68">
         <v>25.774717330933001</v>
       </c>
-      <c r="H68" s="9">
+      <c r="H68">
         <v>60</v>
       </c>
-      <c r="I68" s="9">
+      <c r="I68">
         <v>0.84818619010865004</v>
       </c>
       <c r="O68">
@@ -3120,13 +3120,13 @@
       <c r="D69">
         <v>0.84925543753927002</v>
       </c>
-      <c r="G69" s="9">
+      <c r="G69">
         <v>25.167226791381999</v>
       </c>
-      <c r="H69" s="9">
+      <c r="H69">
         <v>61</v>
       </c>
-      <c r="I69" s="9">
+      <c r="I69">
         <v>0.80111729065305004</v>
       </c>
       <c r="O69">
@@ -3158,13 +3158,13 @@
       <c r="D70">
         <v>0.80731317751798004</v>
       </c>
-      <c r="G70" s="9">
+      <c r="G70">
         <v>25.676012039185</v>
       </c>
-      <c r="H70" s="9">
+      <c r="H70">
         <v>62</v>
       </c>
-      <c r="I70" s="9">
+      <c r="I70">
         <v>0.80730702351251005</v>
       </c>
       <c r="O70">
@@ -3196,13 +3196,13 @@
       <c r="D71">
         <v>0.84779190593383003</v>
       </c>
-      <c r="G71" s="9">
+      <c r="G71">
         <v>25.173902511596999</v>
       </c>
-      <c r="H71" s="9">
+      <c r="H71">
         <v>63</v>
       </c>
-      <c r="I71" s="9">
+      <c r="I71">
         <v>0.84474013035696005</v>
       </c>
       <c r="O71">
@@ -3234,13 +3234,13 @@
       <c r="D72">
         <v>0.82996925343738004</v>
       </c>
-      <c r="G72" s="9">
+      <c r="G72">
         <v>25.755882263183999</v>
       </c>
-      <c r="H72" s="9">
+      <c r="H72">
         <v>64</v>
       </c>
-      <c r="I72" s="9">
+      <c r="I72">
         <v>0.84881083871980001</v>
       </c>
       <c r="O72">
@@ -3272,13 +3272,13 @@
       <c r="D73">
         <v>0.84875558808920004</v>
       </c>
-      <c r="G73" s="9">
+      <c r="G73">
         <v>25.146484375</v>
       </c>
-      <c r="H73" s="9">
+      <c r="H73">
         <v>65</v>
       </c>
-      <c r="I73" s="9">
+      <c r="I73">
         <v>0.83428715641955997</v>
       </c>
       <c r="O73">
@@ -3310,13 +3310,13 @@
       <c r="D74">
         <v>0.80451541391294001</v>
       </c>
-      <c r="G74" s="9">
+      <c r="G74">
         <v>26.771306991576999</v>
       </c>
-      <c r="H74" s="9">
+      <c r="H74">
         <v>66</v>
       </c>
-      <c r="I74" s="9">
+      <c r="I74">
         <v>0.83823967703478997</v>
       </c>
       <c r="O74">
@@ -3348,13 +3348,13 @@
       <c r="D75">
         <v>0.81309401341952003</v>
       </c>
-      <c r="G75" s="9">
+      <c r="G75">
         <v>25.120496749878001</v>
       </c>
-      <c r="H75" s="9">
+      <c r="H75">
         <v>67</v>
       </c>
-      <c r="I75" s="9">
+      <c r="I75">
         <v>0.83837994078772005</v>
       </c>
       <c r="O75">
@@ -3386,13 +3386,13 @@
       <c r="D76">
         <v>0.82139409622232995</v>
       </c>
-      <c r="G76" s="9">
+      <c r="G76">
         <v>25.807857513428001</v>
       </c>
-      <c r="H76" s="9">
+      <c r="H76">
         <v>68</v>
       </c>
-      <c r="I76" s="9">
+      <c r="I76">
         <v>0.80192151783135002</v>
       </c>
       <c r="O76">
@@ -3424,13 +3424,13 @@
       <c r="D77">
         <v>0.77949734258174996</v>
       </c>
-      <c r="G77" s="9">
+      <c r="G77">
         <v>27.316570281981999</v>
       </c>
-      <c r="H77" s="9">
+      <c r="H77">
         <v>69</v>
       </c>
-      <c r="I77" s="9">
+      <c r="I77">
         <v>0.82903958066779004</v>
       </c>
       <c r="O77">
@@ -3462,13 +3462,13 @@
       <c r="D78">
         <v>0.84000133850890002</v>
       </c>
-      <c r="G78" s="9">
+      <c r="G78">
         <v>25.593519210815</v>
       </c>
-      <c r="H78" s="9">
+      <c r="H78">
         <v>70</v>
       </c>
-      <c r="I78" s="9">
+      <c r="I78">
         <v>0.84775192950554001</v>
       </c>
       <c r="O78">
@@ -3500,13 +3500,13 @@
       <c r="D79">
         <v>0.80387419836597995</v>
       </c>
-      <c r="G79" s="9">
+      <c r="G79">
         <v>26.781320571898998</v>
       </c>
-      <c r="H79" s="9">
+      <c r="H79">
         <v>71</v>
       </c>
-      <c r="I79" s="9">
+      <c r="I79">
         <v>0.82852449080498003</v>
       </c>
       <c r="O79">
@@ -3538,13 +3538,13 @@
       <c r="D80">
         <v>0.85094005723179</v>
       </c>
-      <c r="G80" s="9">
+      <c r="G80">
         <v>25.881290435791001</v>
       </c>
-      <c r="H80" s="9">
+      <c r="H80">
         <v>72</v>
       </c>
-      <c r="I80" s="9">
+      <c r="I80">
         <v>0.81308777128644005</v>
       </c>
       <c r="O80">
@@ -3576,13 +3576,13 @@
       <c r="D81">
         <v>0.80403444637068999</v>
       </c>
-      <c r="G81" s="9">
+      <c r="G81">
         <v>28.561592102051002</v>
       </c>
-      <c r="H81" s="9">
+      <c r="H81">
         <v>73</v>
       </c>
-      <c r="I81" s="9">
+      <c r="I81">
         <v>0.81432238726239004</v>
       </c>
       <c r="O81">
@@ -3614,13 +3614,13 @@
       <c r="D82">
         <v>0.81679828326180004</v>
       </c>
-      <c r="G82" s="9">
+      <c r="G82">
         <v>26.592969894408998</v>
       </c>
-      <c r="H82" s="9">
+      <c r="H82">
         <v>74</v>
       </c>
-      <c r="I82" s="9">
+      <c r="I82">
         <v>0.80404940690980997</v>
       </c>
       <c r="O82">
@@ -3649,10 +3649,10 @@
       <c r="D83" t="s">
         <v>9</v>
       </c>
-      <c r="H83" s="9" t="s">
+      <c r="H83" t="s">
         <v>8</v>
       </c>
-      <c r="I83" s="9" t="s">
+      <c r="I83" t="s">
         <v>9</v>
       </c>
       <c r="O83">
@@ -3683,11 +3683,11 @@
         <f>AVERAGE(D8:D82)</f>
         <v>0.82547365727133548</v>
       </c>
-      <c r="G84" s="10">
+      <c r="G84" s="9">
         <f>AVERAGE(G8:G83)</f>
         <v>33.084646860758482</v>
       </c>
-      <c r="I84" s="10">
+      <c r="I84" s="9">
         <f>AVERAGE(I8:I83)</f>
         <v>0.82549496137393674</v>
       </c>
@@ -3731,6 +3731,22 @@
       </c>
     </row>
     <row r="86" spans="2:22">
+      <c r="B86">
+        <f>STDEVA(B8:B82)</f>
+        <v>7059.9943218082017</v>
+      </c>
+      <c r="D86">
+        <f>STDEVA(D8:D82)</f>
+        <v>2.120146844115104E-2</v>
+      </c>
+      <c r="G86">
+        <f>STDEVA(G9:G82)</f>
+        <v>2.0459213613987255</v>
+      </c>
+      <c r="I86">
+        <f>STDEVA(I8:I82)</f>
+        <v>2.120092904111099E-2</v>
+      </c>
       <c r="O86">
         <f>AVERAGE(O10:O84)</f>
         <v>14712.294597625711</v>

</xml_diff>